<commit_message>
fix: Corrigir detecção de sistemas de estrelas no export
PROBLEMA: Lógica errada classificava sistemas de números como estrelas
- Verificava se max(números) <= 12
- Sistemas com números baixos (1,2,3...) eram classificados como estrelas
- Resultado: sheet de estrelas vazia, números misturados

SOLUÇÃO: Verificar pelo NOME do sistema
- Verifica se nome contém 'star' ou 'estrela'
- Mais confiável e correto
- Agora sheet de estrelas terá dados

Isto resolve o bug da sheet de estrelas vazia!
</commit_message>
<xml_diff>
--- a/2-EXCEL/previsao_02012026.xlsx
+++ b/2-EXCEL/previsao_02012026.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F74"/>
   <cols>
     <col min="1" max="1" width="40.83203125" customWidth="1"/>
     <col min="2" max="2" width="50.83203125" customWidth="1"/>
@@ -441,7 +441,7 @@
         <v>7, 8, 9, 13, 17, 19, 22, 24, 25, 26, 28, 30, 31, 32, 35, 37, 38, 39, 40, 41, 42, 43, 44, 45, 47</v>
       </c>
       <c r="E2" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F2" t="str">
         <v>02/01/2026</v>
@@ -461,7 +461,7 @@
         <v>11, 12, 13, 14, 15, 16, 17, 19, 20, 21, 23, 24, 25, 26, 27, 28, 29, 30, 42, 43, 44, 45, 48, 49, 50</v>
       </c>
       <c r="E3" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F3" t="str">
         <v>02/01/2026</v>
@@ -481,7 +481,7 @@
         <v>2, 3, 5, 6, 7, 8</v>
       </c>
       <c r="E4" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F4" t="str">
         <v>02/01/2026</v>
@@ -501,7 +501,7 @@
         <v>6, 7, 8, 9, 10, 11, 12, 18, 19, 20, 21, 22, 27, 28, 29, 30, 33, 34, 35, 36, 37, 42, 43, 44, 45</v>
       </c>
       <c r="E5" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F5" t="str">
         <v>02/01/2026</v>
@@ -521,7 +521,7 @@
         <v>4, 7, 10, 13, 14, 15, 17, 19, 20, 21, 23, 24, 25, 26, 27, 29, 30, 35, 37, 38, 42, 44, 45, 49, 50</v>
       </c>
       <c r="E6" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F6" t="str">
         <v>02/01/2026</v>
@@ -541,7 +541,7 @@
         <v>2, 6, 8, 10, 11, 12</v>
       </c>
       <c r="E7" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F7" t="str">
         <v>02/01/2026</v>
@@ -561,7 +561,7 @@
         <v>7, 10, 13, 14, 15, 17, 19, 20, 21, 23, 24, 25, 26, 27, 29, 30, 35, 37, 38, 39, 42, 44, 45, 48, 50</v>
       </c>
       <c r="E8" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F8" t="str">
         <v>02/01/2026</v>
@@ -581,7 +581,7 @@
         <v>2, 5, 6, 7, 8, 9</v>
       </c>
       <c r="E9" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F9" t="str">
         <v>02/01/2026</v>
@@ -601,7 +601,7 @@
         <v>11, 13, 15, 17, 19, 21, 23, 25, 27, 29, 31, 33, 34, 35, 37, 39, 41, 42, 43, 45, 46, 47, 48, 49, 50</v>
       </c>
       <c r="E10" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F10" t="str">
         <v>02/01/2026</v>
@@ -621,7 +621,7 @@
         <v>3, 6, 7, 12, 13, 14, 16, 17, 19, 20, 21, 23, 24, 25, 27, 28, 30, 35, 37, 38, 39, 47, 48, 49, 50</v>
       </c>
       <c r="E11" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F11" t="str">
         <v>02/01/2026</v>
@@ -641,7 +641,7 @@
         <v>1, 2, 6, 10, 12, 13, 15, 16, 17, 19, 20, 21, 23, 25, 29, 30, 35, 37, 38, 39, 42, 44, 48, 49, 50</v>
       </c>
       <c r="E12" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F12" t="str">
         <v>02/01/2026</v>
@@ -661,7 +661,7 @@
         <v>2, 3, 5, 6, 8, 9</v>
       </c>
       <c r="E13" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F13" t="str">
         <v>02/01/2026</v>
@@ -681,7 +681,7 @@
         <v>3, 4, 5, 8, 9, 10</v>
       </c>
       <c r="E14" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F14" t="str">
         <v>02/01/2026</v>
@@ -701,7 +701,7 @@
         <v>1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25</v>
       </c>
       <c r="E15" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F15" t="str">
         <v>02/01/2026</v>
@@ -721,7 +721,7 @@
         <v>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 21, 22, 23, 24, 25, 26, 28, 29, 31, 32, 34, 41, 42, 44, 45</v>
       </c>
       <c r="E16" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F16" t="str">
         <v>02/01/2026</v>
@@ -741,7 +741,7 @@
         <v>7, 8, 9, 10, 11, 17, 19, 20, 21, 23, 24, 25, 26, 27, 28, 29, 30, 31, 33, 35, 36, 37, 42, 44, 45</v>
       </c>
       <c r="E17" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F17" t="str">
         <v>02/01/2026</v>
@@ -761,7 +761,7 @@
         <v>5, 7, 8, 9, 10, 11, 15, 16, 17, 18, 19, 20, 25, 26, 27, 28, 29, 30, 33, 35, 39, 42, 44, 45, 49</v>
       </c>
       <c r="E18" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F18" t="str">
         <v>02/01/2026</v>
@@ -781,7 +781,7 @@
         <v>2, 5, 7, 8, 9, 11, 16, 17, 18, 24, 25, 27, 28, 29, 31, 32, 33, 35, 36, 39, 40, 41, 45, 46, 49</v>
       </c>
       <c r="E19" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F19" t="str">
         <v>02/01/2026</v>
@@ -801,7 +801,7 @@
         <v>3, 5, 6, 9, 10, 11, 13, 15, 17, 19, 22, 23, 25, 26, 31, 33, 37, 39, 40, 41, 42, 44, 46, 48, 49</v>
       </c>
       <c r="E20" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F20" t="str">
         <v>02/01/2026</v>
@@ -821,7 +821,7 @@
         <v>1, 4, 10, 13, 14, 15, 18, 19, 22, 23, 24, 27, 28, 31, 32, 33, 36, 37, 40, 41, 42, 45, 46, 49, 50</v>
       </c>
       <c r="E21" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F21" t="str">
         <v>02/01/2026</v>
@@ -841,7 +841,7 @@
         <v>7, 8, 9, 10, 11, 19, 20, 21, 22, 23, 27, 28, 29, 30, 31, 33, 34, 35, 36, 37, 42, 43, 44, 45, 46</v>
       </c>
       <c r="E22" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F22" t="str">
         <v>02/01/2026</v>
@@ -861,7 +861,7 @@
         <v>7, 8, 9, 10, 11, 19, 20, 21, 22, 23, 27, 28, 29, 30, 31, 33, 34, 35, 36, 37, 42, 43, 44, 45, 46</v>
       </c>
       <c r="E23" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F23" t="str">
         <v>02/01/2026</v>
@@ -881,7 +881,7 @@
         <v>1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26</v>
       </c>
       <c r="E24" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F24" t="str">
         <v>02/01/2026</v>
@@ -901,7 +901,7 @@
         <v>6, 7, 8, 9, 10, 11, 12, 18, 19, 20, 21, 22, 24, 27, 28, 29, 30, 33, 34, 35, 36, 42, 43, 44, 45</v>
       </c>
       <c r="E25" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F25" t="str">
         <v>02/01/2026</v>
@@ -921,7 +921,7 @@
         <v>4, 7, 10, 12, 13, 15, 17, 19, 20, 21, 24, 25, 26, 27, 29, 30, 34, 35, 37, 38, 39, 42, 44, 45, 49</v>
       </c>
       <c r="E26" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F26" t="str">
         <v>02/01/2026</v>
@@ -941,7 +941,7 @@
         <v>1, 3, 4, 7, 8, 9, 10, 12, 14, 15, 16, 19, 21, 23, 24, 25, 27, 32, 33, 34, 37, 40, 41, 42, 48</v>
       </c>
       <c r="E27" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F27" t="str">
         <v>02/01/2026</v>
@@ -961,7 +961,7 @@
         <v>1, 2, 5, 6, 8, 10, 11, 14, 15, 21, 23, 24, 25, 26, 27, 29, 33, 37, 38, 40, 42, 44, 45, 49, 50</v>
       </c>
       <c r="E28" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F28" t="str">
         <v>02/01/2026</v>
@@ -981,7 +981,7 @@
         <v>1, 2, 5, 8, 9, 10, 11, 14, 15, 17, 22, 23, 24, 26, 27, 29, 31, 33, 37, 40, 42, 44, 45, 49, 50</v>
       </c>
       <c r="E29" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F29" t="str">
         <v>02/01/2026</v>
@@ -1001,7 +1001,7 @@
         <v>2, 3, 4, 5, 9, 10, 11, 14, 15, 21, 23, 24, 25, 29, 30, 31, 33, 35, 36, 40, 42, 44, 45, 49, 50</v>
       </c>
       <c r="E30" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F30" t="str">
         <v>02/01/2026</v>
@@ -1021,7 +1021,7 @@
         <v>1, 3, 5, 7, 9, 11</v>
       </c>
       <c r="E31" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F31" t="str">
         <v>02/01/2026</v>
@@ -1041,7 +1041,7 @@
         <v>6, 7, 8, 9, 10, 11, 12, 18, 19, 20, 21, 22, 23, 24, 26, 27, 28, 29, 30, 31, 32, 33, 34, 35, 36</v>
       </c>
       <c r="E32" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F32" t="str">
         <v>02/01/2026</v>
@@ -1061,7 +1061,7 @@
         <v>1, 2, 3, 4, 5, 6, 10, 11, 12, 14, 15, 16, 18, 20, 21, 23, 27, 29, 33, 34, 36, 46, 48, 49, 50</v>
       </c>
       <c r="E33" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F33" t="str">
         <v>02/01/2026</v>
@@ -1081,7 +1081,7 @@
         <v>1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 18, 22, 31, 32, 33, 34, 35, 36, 37, 38, 39, 40, 41, 46, 47</v>
       </c>
       <c r="E34" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F34" t="str">
         <v>02/01/2026</v>
@@ -1101,7 +1101,7 @@
         <v>1, 4, 9, 10, 11, 12</v>
       </c>
       <c r="E35" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F35" t="str">
         <v>02/01/2026</v>
@@ -1115,13 +1115,13 @@
         <v>Consenso automático entre Anti-Vortex, Média Camadas e Média+3 (Top 25 mais votados)</v>
       </c>
       <c r="C36" t="str">
-        <v>6, 7, 8, 9, 10, 11, 12, 18, 19, 20, 21, 22, 27, 28, 29, 30, 33, 34, 35, 36, 37, 42, 43, 44, 45</v>
+        <v>10, 33, 45, 35, 29, 30, 11, 42, 9, 21</v>
       </c>
       <c r="D36" t="str">
-        <v>1, 2, 3, 4, 5, 13, 14, 15, 16, 17, 23, 24, 25, 26, 31, 32, 38, 39, 40, 41, 46, 47, 48, 49, 50</v>
+        <v>1, 2, 3, 4, 5, 6, 7, 8, 12, 13, 14, 15, 16, 17, 18, 19, 20, 22, 23, 24, 25, 26, 27, 28, 31</v>
       </c>
       <c r="E36" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F36" t="str">
         <v>02/01/2026</v>
@@ -1129,19 +1129,19 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Golden Pair</v>
+        <v>Consensus Auto (Vortex + LSTM + Media3)</v>
       </c>
       <c r="B37" t="str">
-        <v>Aposta nos PARES de estrelas que saem juntos mais frequentemente (Histórico)</v>
+        <v>Consenso automático entre Anti-Vortex, LSTM e Média+3 (Top 25 mais votados)</v>
       </c>
       <c r="C37" t="str">
-        <v>2, 3, 6, 7, 8, 9</v>
+        <v>10, 45, 23, 35, 29, 30, 42, 21, 44, 50</v>
       </c>
       <c r="D37" t="str">
-        <v>1, 4, 5, 10, 11, 12</v>
+        <v>1, 2, 3, 4, 5, 6, 7, 8, 9, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 22, 24, 25, 26, 27, 28</v>
       </c>
       <c r="E37" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F37" t="str">
         <v>02/01/2026</v>
@@ -1149,19 +1149,19 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Hot Numbers</v>
+        <v>Golden Pair</v>
       </c>
       <c r="B38" t="str">
-        <v>Top 10 números mais frequentes nos últimos sorteios</v>
+        <v>Aposta nos PARES de estrelas que saem juntos mais frequentemente (Histórico)</v>
       </c>
       <c r="C38" t="str">
-        <v>44, 23, 42, 19, 29, 21, 17, 50, 10, 25, 37, 45, 20, 35, 15, 27, 26, 7, 13, 38, 14, 24, 30, 49, 4</v>
+        <v>2, 3, 6, 7, 8, 9</v>
       </c>
       <c r="D38" t="str">
-        <v>1, 2, 3, 5, 6, 8, 9, 11, 12, 16, 18, 22, 28, 31, 32, 33, 34, 36, 39, 40, 41, 43, 46, 47, 48</v>
+        <v>1, 4, 5, 10, 11, 12</v>
       </c>
       <c r="E38" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F38" t="str">
         <v>02/01/2026</v>
@@ -1169,19 +1169,19 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Hot Stars</v>
+        <v>Hot Numbers</v>
       </c>
       <c r="B39" t="str">
-        <v>Estrelas mais frequentes nos últimos 50 sorteios</v>
+        <v>Top 10 números mais frequentes nos últimos sorteios</v>
       </c>
       <c r="C39" t="str">
-        <v>2, 10, 12, 5, 6, 8</v>
+        <v>44, 23, 42, 19, 29, 21, 17, 50, 10, 25, 37, 45, 20, 35, 15, 27, 26, 7, 13, 38, 14, 24, 30, 49, 4</v>
       </c>
       <c r="D39" t="str">
-        <v>1, 3, 4, 7, 9, 11</v>
+        <v>1, 2, 3, 5, 6, 8, 9, 11, 12, 16, 18, 22, 28, 31, 32, 33, 34, 36, 39, 40, 41, 43, 46, 47, 48</v>
       </c>
       <c r="E39" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F39" t="str">
         <v>02/01/2026</v>
@@ -1189,19 +1189,19 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>LSTM Neural Net</v>
+        <v>Hot Stars</v>
       </c>
       <c r="B40" t="str">
-        <v>Rede Neuronal Profunda (TensorFlow) com memória de longo prazo.</v>
+        <v>Estrelas mais frequentes nos últimos 50 sorteios</v>
       </c>
       <c r="C40" t="str">
-        <v>42, 35, 20, 23, 17, 29, 21, 19, 45, 44, 10, 48, 14, 50, 30, 27, 15, 25, 13, 38, 26, 37, 24, 39, 7</v>
+        <v>2, 10, 12, 5, 6, 8</v>
       </c>
       <c r="D40" t="str">
-        <v>1, 2, 3, 4, 5, 6, 8, 9, 11, 12, 16, 18, 22, 28, 31, 32, 33, 34, 36, 40, 41, 43, 46, 47, 49</v>
+        <v>1, 3, 4, 7, 9, 11</v>
       </c>
       <c r="E40" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F40" t="str">
         <v>02/01/2026</v>
@@ -1209,19 +1209,19 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Late Stars</v>
+        <v>LSTM Neural Net</v>
       </c>
       <c r="B41" t="str">
-        <v>Estrelas que não saem há mais tempo</v>
+        <v>Rede Neuronal Profunda (TensorFlow) com memória de longo prazo.</v>
       </c>
       <c r="C41" t="str">
-        <v>7, 9, 6, 8, 5, 2</v>
+        <v>44, 42, 25, 21, 23, 10, 29, 30, 17, 45, 38, 19, 15, 35, 50, 37, 7, 27, 20, 16, 4, 49, 48, 14, 39</v>
       </c>
       <c r="D41" t="str">
-        <v>1, 3, 4, 10, 11, 12</v>
+        <v>1, 2, 3, 5, 6, 8, 9, 11, 12, 13, 18, 22, 24, 26, 28, 31, 32, 33, 34, 36, 40, 41, 43, 46, 47</v>
       </c>
       <c r="E41" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F41" t="str">
         <v>02/01/2026</v>
@@ -1229,19 +1229,19 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Machine Learning (Regressão Logística)</v>
+        <v>Late Stars</v>
       </c>
       <c r="B42" t="str">
-        <v>Usa um modelo de classificação binária treinado no histórico recente para prever a probabilidade de cada número.</v>
+        <v>Estrelas que não saem há mais tempo</v>
       </c>
       <c r="C42" t="str">
-        <v>11, 13, 15, 17, 19, 21, 23, 25, 27, 29, 31, 33, 34, 35, 37, 39, 41, 42, 43, 45, 46, 47, 48, 49, 50</v>
+        <v>7, 9, 6, 8, 5, 2</v>
       </c>
       <c r="D42" t="str">
-        <v>1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 12, 14, 16, 18, 20, 22, 24, 26, 28, 30, 32, 36, 38, 40, 44</v>
+        <v>1, 3, 4, 10, 11, 12</v>
       </c>
       <c r="E42" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F42" t="str">
         <v>02/01/2026</v>
@@ -1249,19 +1249,19 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Markov Chain</v>
+        <v>Machine Learning (Regressão Logística)</v>
       </c>
       <c r="B43" t="str">
-        <v>Análise de probabilidades de transição entre números</v>
+        <v>Usa um modelo de classificação binária treinado no histórico recente para prever a probabilidade de cada número.</v>
       </c>
       <c r="C43" t="str">
-        <v>35, 13, 17, 21, 24, 50, 7, 14, 23, 19, 37, 20, 12, 39, 47, 16, 49, 30, 28, 38, 48, 25, 27, 3, 6</v>
+        <v>11, 13, 15, 17, 19, 21, 23, 25, 27, 29, 31, 33, 34, 35, 37, 39, 41, 42, 43, 45, 46, 47, 48, 49, 50</v>
       </c>
       <c r="D43" t="str">
-        <v>1, 2, 4, 5, 8, 9, 10, 11, 15, 18, 22, 26, 29, 31, 32, 33, 34, 36, 40, 41, 42, 43, 44, 45, 46</v>
+        <v>1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 12, 14, 16, 18, 20, 22, 24, 26, 28, 30, 32, 36, 38, 40, 44</v>
       </c>
       <c r="E43" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F43" t="str">
         <v>02/01/2026</v>
@@ -1269,19 +1269,19 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Markov Stars</v>
+        <v>Markov Chain</v>
       </c>
       <c r="B44" t="str">
-        <v>Probabilidade de transição baseada no último sorteio</v>
+        <v>Análise de probabilidades de transição entre números</v>
       </c>
       <c r="C44" t="str">
-        <v>3, 10, 4, 8, 11, 2</v>
+        <v>35, 13, 17, 21, 24, 50, 7, 14, 23, 19, 37, 20, 12, 39, 47, 16, 49, 30, 28, 38, 48, 25, 27, 3, 6</v>
       </c>
       <c r="D44" t="str">
-        <v>1, 5, 6, 7, 9, 12</v>
+        <v>1, 2, 4, 5, 8, 9, 10, 11, 15, 18, 22, 26, 29, 31, 32, 33, 34, 36, 40, 41, 42, 43, 44, 45, 46</v>
       </c>
       <c r="E44" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F44" t="str">
         <v>02/01/2026</v>
@@ -1289,19 +1289,19 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Monte Carlo</v>
+        <v>Markov Stars</v>
       </c>
       <c r="B45" t="str">
-        <v>Simulações probabilísticas para prever números</v>
+        <v>Probabilidade de transição baseada no último sorteio</v>
       </c>
       <c r="C45" t="str">
-        <v>37, 17, 13, 23, 44, 48, 21, 42, 10, 19, 38, 16, 50, 6, 12, 30, 1, 15, 20, 29, 2, 35, 39, 49, 25</v>
+        <v>3, 10, 4, 8, 11, 2</v>
       </c>
       <c r="D45" t="str">
-        <v>3, 4, 5, 7, 8, 9, 11, 14, 18, 22, 24, 26, 27, 28, 31, 32, 33, 34, 36, 40, 41, 43, 45, 46, 47</v>
+        <v>1, 5, 6, 7, 9, 12</v>
       </c>
       <c r="E45" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F45" t="str">
         <v>02/01/2026</v>
@@ -1309,19 +1309,19 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Monte Carlo Stars</v>
+        <v>Monte Carlo</v>
       </c>
       <c r="B46" t="str">
-        <v>Simulações probabilísticas para prever estrelas</v>
+        <v>Simulações probabilísticas para prever números</v>
       </c>
       <c r="C46" t="str">
-        <v>3, 2, 6, 9, 8, 5</v>
+        <v>37, 17, 13, 23, 44, 48, 21, 42, 10, 19, 38, 16, 50, 6, 12, 30, 1, 15, 20, 29, 2, 35, 39, 49, 25</v>
       </c>
       <c r="D46" t="str">
-        <v>1, 4, 7, 10, 11, 12</v>
+        <v>3, 4, 5, 7, 8, 9, 11, 14, 18, 22, 24, 26, 27, 28, 31, 32, 33, 34, 36, 40, 41, 43, 45, 46, 47</v>
       </c>
       <c r="E46" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F46" t="str">
         <v>02/01/2026</v>
@@ -1329,19 +1329,19 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Média +1 Stars</v>
+        <v>Monte Carlo Stars</v>
       </c>
       <c r="B47" t="str">
-        <v>Média dos últimos 50 sorteios + vizinhos (±1) por casa</v>
+        <v>Simulações probabilísticas para prever estrelas</v>
       </c>
       <c r="C47" t="str">
-        <v>3, 4, 5, 8, 9, 10</v>
+        <v>3, 2, 6, 9, 8, 5</v>
       </c>
       <c r="D47" t="str">
-        <v>1, 2, 6, 7, 11, 12</v>
+        <v>1, 4, 7, 10, 11, 12</v>
       </c>
       <c r="E47" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F47" t="str">
         <v>02/01/2026</v>
@@ -1349,19 +1349,19 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>PyramidGaps</v>
+        <v>Média +1 Stars</v>
       </c>
       <c r="B48" t="str">
-        <v>Pirâmide de Dados (Análise de Intervalos)</v>
+        <v>Média dos últimos 50 sorteios + vizinhos (±1) por casa</v>
       </c>
       <c r="C48" t="str">
-        <v>1, 2, 4, 5, 8, 6, 7, 9, 11, 10, 12, 14, 13, 15, 3, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25</v>
+        <v>3, 4, 5, 8, 9, 10</v>
       </c>
       <c r="D48" t="str">
-        <v>26, 27, 28, 29, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 50</v>
+        <v>1, 2, 6, 7, 11, 12</v>
       </c>
       <c r="E48" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F48" t="str">
         <v>02/01/2026</v>
@@ -1369,19 +1369,19 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>PyramidPascal</v>
+        <v>PyramidGaps</v>
       </c>
       <c r="B49" t="str">
-        <v>Pirâmide de Pascal (Soma Mod 10)</v>
+        <v>Pirâmide de Dados (Análise de Intervalos)</v>
       </c>
       <c r="C49" t="str">
-        <v>11, 12, 21, 14, 41, 15, 22, 13, 16, 18, 24, 31, 42, 19, 25, 44, 17, 23, 26, 28, 32, 45, 10, 29, 34</v>
+        <v>1, 2, 4, 5, 8, 6, 7, 9, 11, 10, 12, 14, 13, 15, 3, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25</v>
       </c>
       <c r="D49" t="str">
-        <v>1, 2, 3, 4, 5, 6, 7, 8, 9, 20, 27, 30, 33, 35, 36, 37, 38, 39, 40, 43, 46, 47, 48, 49, 50</v>
+        <v>26, 27, 28, 29, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 50</v>
       </c>
       <c r="E49" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F49" t="str">
         <v>02/01/2026</v>
@@ -1389,19 +1389,19 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Quarteto Complementar</v>
+        <v>PyramidPascal</v>
       </c>
       <c r="B50" t="str">
-        <v>Ensemble de elite com 100% de cobertura (LSTM, Media+3, Random Forest, Média sem as Pontas)</v>
+        <v>Pirâmide de Pascal (Soma Mod 10)</v>
       </c>
       <c r="C50" t="str">
-        <v>35, 29, 27, 7, 20, 23, 21, 19, 45, 10, 30, 24, 9, 8, 11, 28, 31, 36, 33, 42, 17, 44, 25, 26, 37</v>
+        <v>11, 12, 21, 14, 41, 15, 22, 13, 16, 18, 24, 31, 42, 19, 25, 44, 17, 23, 26, 28, 32, 45, 10, 29, 34</v>
       </c>
       <c r="D50" t="str">
-        <v>1, 2, 3, 4, 5, 6, 12, 13, 14, 15, 16, 18, 22, 32, 34, 38, 39, 40, 41, 43, 46, 47, 48, 49, 50</v>
+        <v>1, 2, 3, 4, 5, 6, 7, 8, 9, 20, 27, 30, 33, 35, 36, 37, 38, 39, 40, 43, 46, 47, 48, 49, 50</v>
       </c>
       <c r="E50" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F50" t="str">
         <v>02/01/2026</v>
@@ -1409,19 +1409,19 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Quarteto Elite (LSTM + Media3 + RF + SemPontas)</v>
+        <v>Quarteto Complementar</v>
       </c>
       <c r="B51" t="str">
         <v>Ensemble de elite com 100% de cobertura (LSTM, Media+3, Random Forest, Média sem as Pontas)</v>
       </c>
       <c r="C51" t="str">
-        <v>5, 7, 8, 9, 10, 11, 15, 16, 17, 18, 19, 20, 25, 26, 27, 28, 29, 30, 33, 35, 39, 42, 44, 45, 49</v>
+        <v>29, 35, 7, 27, 21, 23, 10, 30, 45, 19, 20, 9, 8, 11, 28, 31, 36, 33, 44, 42, 25, 17, 37, 16, 49</v>
       </c>
       <c r="D51" t="str">
-        <v>1, 2, 3, 4, 6, 12, 13, 14, 21, 22, 23, 24, 31, 32, 34, 36, 37, 38, 40, 41, 43, 46, 47, 48, 50</v>
+        <v>1, 2, 3, 4, 5, 6, 12, 13, 14, 15, 18, 22, 24, 26, 32, 34, 38, 39, 40, 41, 43, 46, 47, 48, 50</v>
       </c>
       <c r="E51" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F51" t="str">
         <v>02/01/2026</v>
@@ -1429,19 +1429,19 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Random Forest AI</v>
+        <v>Quarteto Elite (LSTM + Media3 + RF + SemPontas)</v>
       </c>
       <c r="B52" t="str">
-        <v>Floresta Aleatória: Ensemble de Árvores de Decisão treinadas em subconjuntos de dados.</v>
+        <v>Ensemble de elite com 100% de cobertura (LSTM, Media+3, Random Forest, Média sem as Pontas)</v>
       </c>
       <c r="C52" t="str">
-        <v>17, 29, 32, 11, 36, 45, 28, 16, 9, 39, 31, 5, 27, 35, 46, 41, 49, 33, 25, 18, 2, 8, 40, 24, 7</v>
+        <v>5, 7, 8, 9, 10, 11, 15, 16, 17, 18, 19, 20, 25, 26, 27, 28, 29, 30, 33, 35, 39, 42, 44, 45, 49</v>
       </c>
       <c r="D52" t="str">
-        <v>1, 3, 4, 6, 10, 12, 13, 14, 15, 19, 20, 21, 22, 23, 26, 30, 34, 37, 38, 42, 43, 44, 47, 48, 50</v>
+        <v>1, 2, 3, 4, 6, 12, 13, 14, 21, 22, 23, 24, 31, 32, 34, 36, 37, 38, 40, 41, 43, 46, 47, 48, 50</v>
       </c>
       <c r="E52" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F52" t="str">
         <v>02/01/2026</v>
@@ -1449,19 +1449,19 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Random Generator</v>
+        <v>Quarteto de Impacto</v>
       </c>
       <c r="B53" t="str">
-        <v>Gerador Aleatório Puro (Baseline Real)</v>
+        <v>Ensemble dinâmico com 212 Jackpots históricos acumulados</v>
       </c>
       <c r="C53" t="str">
-        <v>48, 9, 17, 40, 22, 42, 13, 6, 11, 37, 31, 46, 33, 19, 44, 25, 15, 49, 3, 5, 10, 26, 23, 39, 41</v>
+        <v>13, 25, 41, 42, 24, 44, 9, 14, 6, 21</v>
       </c>
       <c r="D53" t="str">
-        <v>1, 2, 4, 7, 8, 12, 14, 16, 18, 20, 21, 24, 27, 28, 29, 30, 32, 34, 35, 36, 38, 43, 45, 47, 50</v>
+        <v>1, 2, 3, 4, 5, 7, 8, 10, 11, 12, 15, 16, 17, 18, 19, 20, 22, 23, 26, 27, 28, 29, 30, 31, 32</v>
       </c>
       <c r="E53" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F53" t="str">
         <v>02/01/2026</v>
@@ -1469,19 +1469,19 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Root Sum (Raiz Digital)</v>
+        <v>Random Forest AI</v>
       </c>
       <c r="B54" t="str">
-        <v>Agrupa números pela sua Raiz Digital (1-9) e joga nos grupos mais quentes.</v>
+        <v>Floresta Aleatória: Ensemble de Árvores de Decisão treinadas em subconjuntos de dados.</v>
       </c>
       <c r="C54" t="str">
-        <v>4, 37, 36, 10, 19, 28, 14, 23, 15, 24, 33, 1, 13, 31, 40, 32, 41, 50, 42, 18, 27, 45, 46, 22, 49</v>
+        <v>17, 29, 32, 11, 36, 45, 28, 16, 9, 39, 31, 5, 27, 35, 46, 41, 49, 33, 25, 18, 2, 8, 40, 24, 7</v>
       </c>
       <c r="D54" t="str">
-        <v>2, 3, 5, 6, 7, 8, 9, 11, 12, 16, 17, 20, 21, 25, 26, 29, 30, 34, 35, 38, 39, 43, 44, 47, 48</v>
+        <v>1, 3, 4, 6, 10, 12, 13, 14, 15, 19, 20, 21, 22, 23, 26, 30, 34, 37, 38, 42, 43, 44, 47, 48, 50</v>
       </c>
       <c r="E54" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F54" t="str">
         <v>02/01/2026</v>
@@ -1489,19 +1489,19 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Sist Combinado Media+3</v>
+        <v>Random Generator</v>
       </c>
       <c r="B55" t="str">
-        <v>Sistema costumizado criado via Admin UI</v>
+        <v>Gerador Aleatório Puro (Baseline Real)</v>
       </c>
       <c r="C55" t="str">
-        <v>9, 8, 10, 7, 11, 21, 20, 22, 19, 23, 29, 28, 30, 27, 31, 35, 34, 36, 33, 37, 44, 43, 45, 42, 46</v>
+        <v>48, 9, 17, 40, 22, 42, 13, 6, 11, 37, 31, 46, 33, 19, 44, 25, 15, 49, 3, 5, 10, 26, 23, 39, 41</v>
       </c>
       <c r="D55" t="str">
-        <v>1, 2, 3, 4, 5, 6, 12, 13, 14, 15, 16, 17, 18, 24, 25, 26, 32, 38, 39, 40, 41, 47, 48, 49, 50</v>
+        <v>1, 2, 4, 7, 8, 12, 14, 16, 18, 20, 21, 24, 27, 28, 29, 30, 32, 34, 35, 36, 38, 43, 45, 47, 50</v>
       </c>
       <c r="E55" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F55" t="str">
         <v>02/01/2026</v>
@@ -1509,19 +1509,19 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Sist Média + 3 Otimizado</v>
+        <v>Root Sum (Raiz Digital)</v>
       </c>
       <c r="B56" t="str">
-        <v>Média Aparada (Last 10) + 3 Vizinhos com Prioridade à Proximidade</v>
+        <v>Agrupa números pela sua Raiz Digital (1-9) e joga nos grupos mais quentes.</v>
       </c>
       <c r="C56" t="str">
-        <v>29, 44, 9, 21, 35, 8, 34, 20, 22, 30, 36, 43, 10, 28, 45, 7, 11, 27, 33, 37, 42, 46, 19, 23, 31</v>
+        <v>4, 37, 36, 10, 19, 28, 14, 23, 15, 24, 33, 1, 13, 31, 40, 32, 41, 50, 42, 18, 27, 45, 46, 22, 49</v>
       </c>
       <c r="D56" t="str">
-        <v>1, 2, 3, 4, 5, 6, 12, 13, 14, 15, 16, 17, 18, 24, 25, 26, 32, 38, 39, 40, 41, 47, 48, 49, 50</v>
+        <v>2, 3, 5, 6, 7, 8, 9, 11, 12, 16, 17, 20, 21, 25, 26, 29, 30, 34, 35, 38, 39, 43, 44, 47, 48</v>
       </c>
       <c r="E56" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F56" t="str">
         <v>02/01/2026</v>
@@ -1529,19 +1529,19 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Sistema Bronze</v>
+        <v>Sist Combinado Media+3</v>
       </c>
       <c r="B57" t="str">
-        <v>Ensemble dos 9 melhores sistemas (Diversificado)</v>
+        <v>Sistema costumizado criado via Admin UI</v>
       </c>
       <c r="C57" t="str">
-        <v>44, 25, 21, 19, 10, 42, 23, 37, 17, 26, 24, 27, 7, 20, 30, 35, 29, 11, 6, 45, 39, 48, 33, 38, 9</v>
+        <v>9, 8, 10, 7, 11, 21, 20, 22, 19, 23, 29, 28, 30, 27, 31, 35, 34, 36, 33, 37, 44, 43, 45, 42, 46</v>
       </c>
       <c r="D57" t="str">
-        <v>1, 2, 3, 4, 5, 8, 12, 13, 14, 15, 16, 18, 22, 28, 31, 32, 34, 36, 40, 41, 43, 46, 47, 49, 50</v>
+        <v>1, 2, 3, 4, 5, 6, 12, 13, 14, 15, 16, 17, 18, 24, 25, 26, 32, 38, 39, 40, 41, 47, 48, 49, 50</v>
       </c>
       <c r="E57" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F57" t="str">
         <v>02/01/2026</v>
@@ -1549,19 +1549,19 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Sistema Elástico</v>
+        <v>Sist Média + 3 Otimizado</v>
       </c>
       <c r="B58" t="str">
-        <v>Baseado na Regressão à Média (Força Elástica)</v>
+        <v>Média Aparada (Last 10) + 3 Vizinhos com Prioridade à Proximidade</v>
       </c>
       <c r="C58" t="str">
-        <v>10, 9, 4, 2, 6, 1, 11, 7, 5, 8, 3, 21, 16, 17, 19, 20, 14, 25, 23, 13, 15, 24, 26, 18, 22</v>
+        <v>29, 44, 9, 21, 35, 8, 34, 20, 22, 30, 36, 43, 10, 28, 45, 7, 11, 27, 33, 37, 42, 46, 19, 23, 31</v>
       </c>
       <c r="D58" t="str">
-        <v>12, 27, 28, 29, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 50</v>
+        <v>1, 2, 3, 4, 5, 6, 12, 13, 14, 15, 16, 17, 18, 24, 25, 26, 32, 38, 39, 40, 41, 47, 48, 49, 50</v>
       </c>
       <c r="E58" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F58" t="str">
         <v>02/01/2026</v>
@@ -1569,19 +1569,19 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Sistema Média Camadas</v>
+        <v>Sistema Bronze</v>
       </c>
       <c r="B59" t="str">
-        <v>Média + 3 com Camadas de Equilíbrio Estatístico (55% Acc)</v>
+        <v>Ensemble dos 9 melhores sistemas (Diversificado)</v>
       </c>
       <c r="C59" t="str">
-        <v>21, 35, 30, 45, 9, 42, 10, 20, 28, 36, 29, 44, 7, 27, 33, 8, 22, 34, 43, 6, 12, 18, 24, 11, 19</v>
+        <v>44, 25, 21, 6, 19, 10, 42, 23, 37, 49, 17, 39, 48, 27, 7, 20, 30, 35, 29, 38, 11, 15, 45, 14, 50</v>
       </c>
       <c r="D59" t="str">
-        <v>1, 2, 3, 4, 5, 13, 14, 15, 16, 17, 23, 25, 26, 31, 32, 37, 38, 39, 40, 41, 46, 47, 48, 49, 50</v>
+        <v>1, 2, 3, 4, 5, 8, 9, 12, 13, 16, 18, 22, 24, 26, 28, 31, 32, 33, 34, 36, 40, 41, 43, 46, 47</v>
       </c>
       <c r="E59" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F59" t="str">
         <v>02/01/2026</v>
@@ -1589,19 +1589,19 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Sistema Média Vizinhos</v>
+        <v>Sistema Elástico</v>
       </c>
       <c r="B60" t="str">
-        <v>Estratégia fixa: Média por casa + Vizinhos (25 números)</v>
+        <v>Baseado na Regressão à Média (Força Elástica)</v>
       </c>
       <c r="C60" t="str">
-        <v>6, 7, 8, 9, 10, 14, 15, 16, 17, 18, 23, 24, 25, 26, 27, 32, 33, 34, 35, 36, 41, 42, 43, 44, 45</v>
+        <v>10, 9, 4, 2, 6, 1, 11, 7, 5, 8, 3, 21, 16, 17, 19, 20, 14, 25, 23, 13, 15, 24, 26, 18, 22</v>
       </c>
       <c r="D60" t="str">
-        <v>1, 2, 3, 4, 5, 11, 12, 13, 19, 20, 21, 22, 28, 29, 30, 31, 37, 38, 39, 40, 46, 47, 48, 49, 50</v>
+        <v>12, 27, 28, 29, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 50</v>
       </c>
       <c r="E60" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F60" t="str">
         <v>02/01/2026</v>
@@ -1609,19 +1609,19 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Sistema Oscilação Universal V2</v>
+        <v>Sistema Média Camadas</v>
       </c>
       <c r="B61" t="str">
-        <v>Previsão direta de oscilação baseada em raiz dominante</v>
+        <v>Média + 3 com Camadas de Equilíbrio Estatístico (55% Acc)</v>
       </c>
       <c r="C61" t="str">
-        <v>44, 42, 19, 29, 21, 17, 10, 25, 37, 45, 20, 35, 15, 27, 26, 7, 13, 38, 24, 30, 49, 4, 12, 34, 39</v>
+        <v>21, 35, 30, 45, 9, 42, 10, 20, 28, 36, 29, 44, 7, 27, 33, 8, 22, 34, 43, 6, 12, 18, 24, 11, 19</v>
       </c>
       <c r="D61" t="str">
-        <v>1, 2, 3, 5, 6, 8, 9, 11, 14, 16, 18, 22, 23, 28, 31, 32, 33, 36, 40, 41, 43, 46, 47, 48, 50</v>
+        <v>1, 2, 3, 4, 5, 13, 14, 15, 16, 17, 23, 25, 26, 31, 32, 37, 38, 39, 40, 41, 46, 47, 48, 49, 50</v>
       </c>
       <c r="E61" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F61" t="str">
         <v>02/01/2026</v>
@@ -1629,19 +1629,19 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Sistema Ouro</v>
+        <v>Sistema Média Vizinhos</v>
       </c>
       <c r="B62" t="str">
-        <v>Ensemble dos 3 melhores sistemas (Elite)</v>
+        <v>Estratégia fixa: Média por casa + Vizinhos (25 números)</v>
       </c>
       <c r="C62" t="str">
-        <v>10, 17, 19, 23, 25, 26, 37, 42, 44, 7, 20, 21, 24, 27, 29, 30, 35, 45, 13, 15, 39, 48, 9, 11, 31</v>
+        <v>6, 7, 8, 9, 10, 14, 15, 16, 17, 18, 23, 24, 25, 26, 27, 32, 33, 34, 35, 36, 41, 42, 43, 44, 45</v>
       </c>
       <c r="D62" t="str">
-        <v>1, 2, 3, 4, 5, 6, 8, 12, 14, 16, 18, 22, 28, 32, 33, 34, 36, 38, 40, 41, 43, 46, 47, 49, 50</v>
+        <v>1, 2, 3, 4, 5, 11, 12, 13, 19, 20, 21, 22, 28, 29, 30, 31, 37, 38, 39, 40, 46, 47, 48, 49, 50</v>
       </c>
       <c r="E62" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F62" t="str">
         <v>02/01/2026</v>
@@ -1649,19 +1649,19 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Sistema Platina</v>
+        <v>Sistema Oscilação Universal V2</v>
       </c>
       <c r="B63" t="str">
-        <v>Ensemble dos 12 melhores sistemas (Abrangente)</v>
+        <v>Previsão direta de oscilação baseada em raiz dominante</v>
       </c>
       <c r="C63" t="str">
-        <v>21, 19, 44, 42, 37, 27, 35, 29, 11, 25, 10, 23, 7, 20, 30, 45, 33, 17, 9, 6, 8, 26, 24, 39, 48</v>
+        <v>44, 42, 19, 29, 21, 17, 10, 25, 37, 45, 20, 35, 15, 27, 26, 7, 13, 38, 24, 30, 49, 4, 12, 34, 39</v>
       </c>
       <c r="D63" t="str">
-        <v>1, 2, 3, 4, 5, 12, 13, 14, 15, 16, 18, 22, 28, 31, 32, 34, 36, 38, 40, 41, 43, 46, 47, 49, 50</v>
+        <v>1, 2, 3, 5, 6, 8, 9, 11, 14, 16, 18, 22, 23, 28, 31, 32, 33, 36, 40, 41, 43, 46, 47, 48, 50</v>
       </c>
       <c r="E63" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F63" t="str">
         <v>02/01/2026</v>
@@ -1669,19 +1669,19 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Sistema Prata</v>
+        <v>Sistema Ouro</v>
       </c>
       <c r="B64" t="str">
-        <v>Ensemble dos 6 melhores sistemas (Equilibrado)</v>
+        <v>Ensemble dos 3 melhores sistemas (Elite)</v>
       </c>
       <c r="C64" t="str">
-        <v>10, 19, 42, 44, 17, 23, 25, 26, 37, 7, 20, 21, 24, 27, 29, 30, 35, 45, 9, 11, 33, 13, 15, 39, 48</v>
+        <v>10, 15, 17, 19, 23, 25, 37, 39, 42, 44, 48, 49, 4, 7, 14, 16, 20, 21, 27, 29, 30, 35, 38, 45, 50</v>
       </c>
       <c r="D64" t="str">
-        <v>1, 2, 3, 4, 5, 6, 8, 12, 14, 16, 18, 22, 28, 31, 32, 34, 36, 38, 40, 41, 43, 46, 47, 49, 50</v>
+        <v>1, 2, 3, 5, 6, 8, 9, 11, 12, 13, 18, 22, 24, 26, 28, 31, 32, 33, 34, 36, 40, 41, 43, 46, 47</v>
       </c>
       <c r="E64" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F64" t="str">
         <v>02/01/2026</v>
@@ -1689,19 +1689,19 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Standard Deviation</v>
+        <v>Sistema Platina</v>
       </c>
       <c r="B65" t="str">
-        <v>Estatística Posicional: Usa a Média e Desvio Padrão de cada posição (1ª a 5ª bola) para encontrar alvos.</v>
+        <v>Ensemble dos 12 melhores sistemas (Abrangente)</v>
       </c>
       <c r="C65" t="str">
-        <v>8, 7, 9, 15, 1, 14, 16, 23, 24, 25, 32, 33, 34, 42, 41, 40, 48, 10, 4, 27, 37, 12, 19, 21, 3</v>
+        <v>21, 19, 44, 25, 42, 23, 37, 27, 35, 29, 11, 10, 49, 17, 39, 48, 7, 20, 30, 45, 6, 33, 15, 38, 50</v>
       </c>
       <c r="D65" t="str">
-        <v>2, 5, 6, 11, 13, 17, 18, 20, 22, 26, 28, 29, 30, 31, 35, 36, 38, 39, 43, 44, 45, 46, 47, 49, 50</v>
+        <v>1, 2, 3, 4, 5, 8, 9, 12, 13, 14, 16, 18, 22, 24, 26, 28, 31, 32, 34, 36, 40, 41, 43, 46, 47</v>
       </c>
       <c r="E65" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F65" t="str">
         <v>02/01/2026</v>
@@ -1709,19 +1709,19 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Star LSTM Neural Net</v>
+        <v>Sistema Prata</v>
       </c>
       <c r="B66" t="str">
-        <v>Rede Neuronal (LSTM) especializada em prever Estrelas (1-12).</v>
+        <v>Ensemble dos 6 melhores sistemas (Equilibrado)</v>
       </c>
       <c r="C66" t="str">
-        <v>2, 3, 7, 9, 8, 1</v>
+        <v>10, 19, 42, 44, 15, 17, 23, 25, 37, 39, 48, 49, 7, 20, 21, 27, 29, 30, 35, 45, 6, 9, 11, 22, 33</v>
       </c>
       <c r="D66" t="str">
-        <v>4, 5, 6, 10, 11, 12</v>
+        <v>1, 2, 3, 4, 5, 8, 12, 13, 14, 16, 18, 24, 26, 28, 31, 32, 34, 36, 38, 40, 41, 43, 46, 47, 50</v>
       </c>
       <c r="E66" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F66" t="str">
         <v>02/01/2026</v>
@@ -1729,19 +1729,19 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>Star Platinum</v>
+        <v>Standard Deviation</v>
       </c>
       <c r="B67" t="str">
-        <v>Ensemble ponderado dos melhores sistemas de estrelas</v>
+        <v>Estatística Posicional: Usa a Média e Desvio Padrão de cada posição (1ª a 5ª bola) para encontrar alvos.</v>
       </c>
       <c r="C67" t="str">
-        <v>10, 2, 8, 3, 6, 7</v>
+        <v>8, 7, 9, 15, 1, 14, 16, 23, 24, 25, 32, 33, 34, 42, 41, 40, 48, 10, 4, 27, 37, 12, 19, 21, 3</v>
       </c>
       <c r="D67" t="str">
-        <v>1, 4, 5, 9, 11, 12</v>
+        <v>2, 5, 6, 11, 13, 17, 18, 20, 22, 26, 28, 29, 30, 31, 35, 36, 38, 39, 43, 44, 45, 46, 47, 49, 50</v>
       </c>
       <c r="E67" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F67" t="str">
         <v>02/01/2026</v>
@@ -1749,19 +1749,19 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Vortex Multi-Canal (2 canais)</v>
+        <v>Star LSTM Neural Net</v>
       </c>
       <c r="B68" t="str">
-        <v>Vortex com 2 linhas diagonais (canais de energia)</v>
+        <v>Rede Neuronal (LSTM) especializada em prever Estrelas (1-12).</v>
       </c>
       <c r="C68" t="str">
-        <v>33, 15, 24, 11, 10, 23, 26, 40, 50, 1, 25, 29, 27, 45, 8, 37, 49, 5, 2, 14, 21, 44, 42, 38, 6</v>
+        <v>2, 3, 7, 9, 8, 1</v>
       </c>
       <c r="D68" t="str">
-        <v>3, 4, 7, 9, 12, 13, 16, 17, 18, 19, 20, 22, 28, 30, 31, 32, 34, 35, 36, 39, 41, 43, 46, 47, 48</v>
+        <v>4, 5, 6, 10, 11, 12</v>
       </c>
       <c r="E68" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F68" t="str">
         <v>02/01/2026</v>
@@ -1769,19 +1769,19 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Vortex Multi-Canal (3 canais)</v>
+        <v>Star Platinum</v>
       </c>
       <c r="B69" t="str">
-        <v>Vortex com 3 linhas diagonais (canais de energia)</v>
+        <v>Ensemble ponderado dos melhores sistemas de estrelas</v>
       </c>
       <c r="C69" t="str">
-        <v>45, 29, 10, 33, 11, 15, 40, 24, 27, 50, 5, 23, 37, 17, 44, 31, 42, 26, 2, 9, 8, 14, 49, 1, 22</v>
+        <v>10, 2, 8, 3, 6, 7</v>
       </c>
       <c r="D69" t="str">
-        <v>3, 4, 6, 7, 12, 13, 16, 18, 19, 20, 21, 25, 28, 30, 32, 34, 35, 36, 38, 39, 41, 43, 46, 47, 48</v>
+        <v>1, 4, 5, 9, 11, 12</v>
       </c>
       <c r="E69" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F69" t="str">
         <v>02/01/2026</v>
@@ -1789,19 +1789,19 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Vortex Pyramid</v>
+        <v>Vortex Multi-Canal (2 canais)</v>
       </c>
       <c r="B70" t="str">
-        <v>Pirâmide Vortex (Cálculo Toroidal/Cilíndrico)</v>
+        <v>Vortex com 2 linhas diagonais (canais de energia)</v>
       </c>
       <c r="C70" t="str">
-        <v>50, 10, 33, 2, 45, 23, 25, 35, 29, 30, 11, 14, 24, 31, 49, 4, 15, 42, 9, 21, 36, 44, 3, 40, 5</v>
+        <v>33, 15, 24, 11, 10, 23, 26, 40, 50, 1, 25, 29, 27, 45, 8, 37, 49, 5, 2, 14, 21, 44, 42, 38, 6</v>
       </c>
       <c r="D70" t="str">
-        <v>1, 6, 7, 8, 12, 13, 16, 17, 18, 19, 20, 22, 26, 27, 28, 32, 34, 37, 38, 39, 41, 43, 46, 47, 48</v>
+        <v>3, 4, 7, 9, 12, 13, 16, 17, 18, 19, 20, 22, 28, 30, 31, 32, 34, 35, 36, 39, 41, 43, 46, 47, 48</v>
       </c>
       <c r="E70" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F70" t="str">
         <v>02/01/2026</v>
@@ -1809,19 +1809,19 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Vortex Stars</v>
+        <v>Vortex Multi-Canal (3 canais)</v>
       </c>
       <c r="B71" t="str">
-        <v>Sistema Vortex adaptado para estrelas (Ressonância Toroidal)</v>
+        <v>Vortex com 3 linhas diagonais (canais de energia)</v>
       </c>
       <c r="C71" t="str">
-        <v>1, 9, 11, 7, 5, 3</v>
+        <v>45, 29, 10, 33, 11, 15, 40, 24, 27, 50, 5, 23, 37, 17, 44, 31, 42, 26, 2, 9, 8, 14, 49, 1, 22</v>
       </c>
       <c r="D71" t="str">
-        <v>2, 4, 6, 8, 10, 12</v>
+        <v>3, 4, 6, 7, 12, 13, 16, 18, 19, 20, 21, 25, 28, 30, 32, 34, 35, 36, 38, 39, 41, 43, 46, 47, 48</v>
       </c>
       <c r="E71" t="str">
-        <v>31/12/2025</v>
+        <v>01/01/2026</v>
       </c>
       <c r="F71" t="str">
         <v>02/01/2026</v>
@@ -1829,27 +1829,67 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
+        <v>Vortex Pyramid</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Pirâmide Vortex (Cálculo Toroidal/Cilíndrico)</v>
+      </c>
+      <c r="C72" t="str">
+        <v>50, 10, 33, 2, 45, 23, 25, 35, 29, 30, 11, 14, 24, 31, 49, 4, 15, 42, 9, 21, 36, 44, 3, 40, 5</v>
+      </c>
+      <c r="D72" t="str">
+        <v>1, 6, 7, 8, 12, 13, 16, 17, 18, 19, 20, 22, 26, 27, 28, 32, 34, 37, 38, 39, 41, 43, 46, 47, 48</v>
+      </c>
+      <c r="E72" t="str">
+        <v>01/01/2026</v>
+      </c>
+      <c r="F72" t="str">
+        <v>02/01/2026</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>Vortex Stars</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Sistema Vortex adaptado para estrelas (Ressonância Toroidal)</v>
+      </c>
+      <c r="C73" t="str">
+        <v>1, 9, 11, 7, 5, 3</v>
+      </c>
+      <c r="D73" t="str">
+        <v>2, 4, 6, 8, 10, 12</v>
+      </c>
+      <c r="E73" t="str">
+        <v>01/01/2026</v>
+      </c>
+      <c r="F73" t="str">
+        <v>02/01/2026</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
         <v>média sem as pontas</v>
       </c>
-      <c r="B72" t="str">
+      <c r="B74" t="str">
         <v>Média aparada (sem extremos) por posição nos últimos 10 sorteios</v>
       </c>
-      <c r="C72" t="str">
+      <c r="C74" t="str">
         <v>6, 7, 8, 9, 10, 11, 12, 18, 19, 20, 21, 22, 23, 24, 26, 27, 28, 29, 30, 31, 32, 33, 34, 35, 36</v>
       </c>
-      <c r="D72" t="str">
+      <c r="D74" t="str">
         <v>1, 2, 3, 4, 5, 13, 14, 15, 16, 17, 25, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 50</v>
       </c>
-      <c r="E72" t="str">
-        <v>31/12/2025</v>
-      </c>
-      <c r="F72" t="str">
+      <c r="E74" t="str">
+        <v>01/01/2026</v>
+      </c>
+      <c r="F74" t="str">
         <v>02/01/2026</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F72"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F74"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: Medal Systems ordenacao bug
</commit_message>
<xml_diff>
--- a/2-EXCEL/previsao_02012026.xlsx
+++ b/2-EXCEL/previsao_02012026.xlsx
@@ -1135,10 +1135,10 @@
         <v>Consenso automático entre Anti-Vortex, LSTM e Média+3 (Top 25 mais votados)</v>
       </c>
       <c r="C37" t="str">
-        <v>10, 45, 23, 35, 29, 30, 42, 21, 44, 50</v>
+        <v>10, 45, 23, 35, 29, 30, 42, 9, 21, 44</v>
       </c>
       <c r="D37" t="str">
-        <v>1, 2, 3, 4, 5, 6, 7, 8, 9, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 22, 24, 25, 26, 27, 28</v>
+        <v>1, 2, 3, 4, 5, 6, 7, 8, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 22, 24, 25, 26, 27, 28, 31</v>
       </c>
       <c r="E37" t="str">
         <v>01/01/2026</v>
@@ -1215,10 +1215,10 @@
         <v>Rede Neuronal Profunda (TensorFlow) com memória de longo prazo.</v>
       </c>
       <c r="C41" t="str">
-        <v>44, 42, 25, 21, 23, 10, 29, 30, 17, 45, 38, 19, 15, 35, 50, 37, 7, 27, 20, 16, 4, 49, 48, 14, 39</v>
+        <v>42, 29, 13, 50, 10, 25, 17, 19, 44, 45, 28, 35, 7, 21, 48, 14, 49, 5, 23, 15, 9, 34, 30, 3, 26</v>
       </c>
       <c r="D41" t="str">
-        <v>1, 2, 3, 5, 6, 8, 9, 11, 12, 13, 18, 22, 24, 26, 28, 31, 32, 33, 34, 36, 40, 41, 43, 46, 47</v>
+        <v>1, 2, 4, 6, 8, 11, 12, 16, 18, 20, 22, 24, 27, 31, 32, 33, 36, 37, 38, 39, 40, 41, 43, 46, 47</v>
       </c>
       <c r="E41" t="str">
         <v>01/01/2026</v>
@@ -1415,10 +1415,10 @@
         <v>Ensemble de elite com 100% de cobertura (LSTM, Media+3, Random Forest, Média sem as Pontas)</v>
       </c>
       <c r="C51" t="str">
-        <v>29, 35, 7, 27, 21, 23, 10, 30, 45, 19, 20, 9, 8, 11, 28, 31, 36, 33, 44, 42, 25, 17, 37, 16, 49</v>
+        <v>29, 28, 35, 7, 9, 10, 19, 45, 21, 23, 34, 30, 8, 11, 27, 31, 36, 33, 42, 25, 17, 44, 49, 5, 26</v>
       </c>
       <c r="D51" t="str">
-        <v>1, 2, 3, 4, 5, 6, 12, 13, 14, 15, 18, 22, 24, 26, 32, 34, 38, 39, 40, 41, 43, 46, 47, 48, 50</v>
+        <v>1, 2, 3, 4, 6, 12, 13, 14, 15, 16, 18, 20, 22, 24, 32, 37, 38, 39, 40, 41, 43, 46, 47, 48, 50</v>
       </c>
       <c r="E51" t="str">
         <v>01/01/2026</v>
@@ -1575,10 +1575,10 @@
         <v>Ensemble dos 9 melhores sistemas (Diversificado)</v>
       </c>
       <c r="C59" t="str">
-        <v>44, 25, 21, 6, 19, 10, 42, 23, 37, 49, 17, 39, 48, 27, 7, 20, 30, 35, 29, 38, 11, 15, 45, 14, 50</v>
+        <v>44, 25, 21, 6, 19, 10, 42, 23, 49, 9, 3, 17, 48, 5, 26, 7, 30, 35, 29, 11, 13, 15, 28, 45, 14</v>
       </c>
       <c r="D59" t="str">
-        <v>1, 2, 3, 4, 5, 8, 9, 12, 13, 16, 18, 22, 24, 26, 28, 31, 32, 33, 34, 36, 40, 41, 43, 46, 47</v>
+        <v>1, 2, 4, 8, 12, 16, 18, 20, 22, 24, 27, 31, 32, 33, 34, 36, 37, 38, 39, 40, 41, 43, 46, 47, 50</v>
       </c>
       <c r="E59" t="str">
         <v>01/01/2026</v>
@@ -1675,10 +1675,10 @@
         <v>Ensemble dos 3 melhores sistemas (Elite)</v>
       </c>
       <c r="C64" t="str">
-        <v>10, 15, 17, 19, 23, 25, 37, 39, 42, 44, 48, 49, 4, 7, 14, 16, 20, 21, 27, 29, 30, 35, 38, 45, 50</v>
+        <v>3, 5, 9, 10, 13, 15, 17, 19, 23, 25, 26, 42, 44, 48, 49, 7, 14, 21, 28, 29, 30, 34, 35, 45, 50</v>
       </c>
       <c r="D64" t="str">
-        <v>1, 2, 3, 5, 6, 8, 9, 11, 12, 13, 18, 22, 24, 26, 28, 31, 32, 33, 34, 36, 40, 41, 43, 46, 47</v>
+        <v>1, 2, 4, 6, 8, 11, 12, 16, 18, 20, 22, 24, 27, 31, 32, 33, 36, 37, 38, 39, 40, 41, 43, 46, 47</v>
       </c>
       <c r="E64" t="str">
         <v>01/01/2026</v>
@@ -1695,10 +1695,10 @@
         <v>Ensemble dos 12 melhores sistemas (Abrangente)</v>
       </c>
       <c r="C65" t="str">
-        <v>21, 19, 44, 25, 42, 23, 37, 27, 35, 29, 11, 10, 49, 17, 39, 48, 7, 20, 30, 45, 6, 33, 15, 38, 50</v>
+        <v>21, 19, 44, 25, 42, 23, 35, 29, 11, 10, 49, 9, 17, 48, 7, 30, 45, 34, 6, 33, 37, 27, 3, 13, 5</v>
       </c>
       <c r="D65" t="str">
-        <v>1, 2, 3, 4, 5, 8, 9, 12, 13, 14, 16, 18, 22, 24, 26, 28, 31, 32, 34, 36, 40, 41, 43, 46, 47</v>
+        <v>1, 2, 4, 8, 12, 14, 15, 16, 18, 20, 22, 24, 26, 28, 31, 32, 36, 38, 39, 40, 41, 43, 46, 47, 50</v>
       </c>
       <c r="E65" t="str">
         <v>01/01/2026</v>
@@ -1715,10 +1715,10 @@
         <v>Ensemble dos 6 melhores sistemas (Equilibrado)</v>
       </c>
       <c r="C66" t="str">
-        <v>10, 19, 42, 44, 15, 17, 23, 25, 37, 39, 48, 49, 7, 20, 21, 27, 29, 30, 35, 45, 6, 9, 11, 22, 33</v>
+        <v>9, 10, 19, 42, 44, 3, 5, 13, 15, 17, 23, 25, 26, 48, 49, 7, 21, 28, 29, 30, 34, 35, 45, 6, 11</v>
       </c>
       <c r="D66" t="str">
-        <v>1, 2, 3, 4, 5, 8, 12, 13, 14, 16, 18, 24, 26, 28, 31, 32, 34, 36, 38, 40, 41, 43, 46, 47, 50</v>
+        <v>1, 2, 4, 8, 12, 14, 16, 18, 20, 22, 24, 27, 31, 32, 33, 36, 37, 38, 39, 40, 41, 43, 46, 47, 50</v>
       </c>
       <c r="E66" t="str">
         <v>01/01/2026</v>

</xml_diff>